<commit_message>
Updated resource references to point to 314e profiles
</commit_message>
<xml_diff>
--- a/314e-ig/output/StructureDefinition-observation-lab-general-314e.xlsx
+++ b/314e-ig/output/StructureDefinition-observation-lab-general-314e.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="597">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3135" uniqueCount="598">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-05-26T12:06:33+05:30</t>
+    <t>2026-05-26T19:54:55+05:30</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1759,6 +1759,10 @@
   </si>
   <si>
     <t>childObservation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(http://314e.com/fhir/StructureDefinition/observation-lab-general-314e) {http://314e.com/fhir/StructureDefinition/reference-314e}
+</t>
   </si>
   <si>
     <t>Observation.derivedFrom</t>
@@ -9653,7 +9657,7 @@
         <v>93</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>538</v>
+        <v>547</v>
       </c>
       <c r="L62" t="s" s="2">
         <v>539</v>
@@ -9747,10 +9751,10 @@
     </row>
     <row r="63" hidden="true">
       <c r="A63" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -9773,16 +9777,16 @@
         <v>93</v>
       </c>
       <c r="K63" t="s" s="2">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="N63" t="s" s="2">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
@@ -9832,7 +9836,7 @@
         <v>20</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="AG63" t="s" s="2">
         <v>80</v>
@@ -9856,7 +9860,7 @@
         <v>543</v>
       </c>
       <c r="AN63" t="s" s="2">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="AO63" t="s" s="2">
         <v>20</v>
@@ -9867,10 +9871,10 @@
     </row>
     <row r="64" hidden="true">
       <c r="A64" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
@@ -9896,16 +9900,16 @@
         <v>484</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="N64" t="s" s="2">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="O64" t="s" s="2">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="P64" t="s" s="2">
         <v>20</v>
@@ -9954,7 +9958,7 @@
         <v>20</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>80</v>
@@ -9975,10 +9979,10 @@
         <v>20</v>
       </c>
       <c r="AM64" t="s" s="2">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="AN64" t="s" s="2">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="AO64" t="s" s="2">
         <v>20</v>
@@ -9989,10 +9993,10 @@
     </row>
     <row r="65" hidden="true">
       <c r="A65" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
@@ -10107,10 +10111,10 @@
     </row>
     <row r="66" hidden="true">
       <c r="A66" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
@@ -10227,10 +10231,10 @@
     </row>
     <row r="67" hidden="true">
       <c r="A67" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
@@ -10349,10 +10353,10 @@
     </row>
     <row r="68" hidden="true">
       <c r="A68" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -10378,13 +10382,13 @@
         <v>238</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="N68" t="s" s="2">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="O68" t="s" s="2">
         <v>338</v>
@@ -10415,10 +10419,10 @@
         <v>158</v>
       </c>
       <c r="Y68" t="s" s="2">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="Z68" t="s" s="2">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="AA68" t="s" s="2">
         <v>20</v>
@@ -10436,7 +10440,7 @@
         <v>20</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="AG68" t="s" s="2">
         <v>92</v>
@@ -10454,7 +10458,7 @@
         <v>20</v>
       </c>
       <c r="AL68" t="s" s="2">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="AM68" t="s" s="2">
         <v>343</v>
@@ -10471,10 +10475,10 @@
     </row>
     <row r="69" hidden="true">
       <c r="A69" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -10500,13 +10504,13 @@
         <v>405</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="N69" t="s" s="2">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="O69" t="s" s="2">
         <v>409</v>
@@ -10558,7 +10562,7 @@
         <v>20</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>80</v>
@@ -10576,7 +10580,7 @@
         <v>20</v>
       </c>
       <c r="AL69" t="s" s="2">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="AM69" t="s" s="2">
         <v>413</v>
@@ -10593,10 +10597,10 @@
     </row>
     <row r="70" hidden="true">
       <c r="A70" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
@@ -10622,13 +10626,13 @@
         <v>417</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="N70" t="s" s="2">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="O70" t="s" s="2">
         <v>421</v>
@@ -10680,7 +10684,7 @@
         <v>20</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>80</v>
@@ -10689,7 +10693,7 @@
         <v>92</v>
       </c>
       <c r="AI70" t="s" s="2">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="AJ70" t="s" s="2">
         <v>104</v>
@@ -10715,10 +10719,10 @@
     </row>
     <row r="71" hidden="true">
       <c r="A71" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
@@ -10744,7 +10748,7 @@
         <v>238</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="M71" t="s" s="2">
         <v>429</v>
@@ -10802,7 +10806,7 @@
         <v>20</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>80</v>
@@ -10837,10 +10841,10 @@
     </row>
     <row r="72" hidden="true">
       <c r="A72" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
@@ -10866,13 +10870,13 @@
         <v>484</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="N72" t="s" s="2">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="O72" t="s" s="2">
         <v>488</v>
@@ -10924,7 +10928,7 @@
         <v>20</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>80</v>
@@ -10959,10 +10963,10 @@
     </row>
     <row r="73" hidden="true">
       <c r="A73" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -11077,10 +11081,10 @@
     </row>
     <row r="74" hidden="true">
       <c r="A74" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -11197,10 +11201,10 @@
     </row>
     <row r="75" hidden="true">
       <c r="A75" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -11319,10 +11323,10 @@
     </row>
     <row r="76" hidden="true">
       <c r="A76" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -11437,10 +11441,10 @@
     </row>
     <row r="77" hidden="true">
       <c r="A77" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
@@ -11555,10 +11559,10 @@
     </row>
     <row r="78" hidden="true">
       <c r="A78" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
@@ -11624,7 +11628,7 @@
         <v>516</v>
       </c>
       <c r="Z78" t="s" s="2">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="AA78" t="s" s="2">
         <v>20</v>
@@ -11677,10 +11681,10 @@
     </row>
     <row r="79" hidden="true">
       <c r="A79" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B79" t="s" s="2">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="C79" s="2"/>
       <c r="D79" t="s" s="2">
@@ -11746,7 +11750,7 @@
         <v>525</v>
       </c>
       <c r="Z79" t="s" s="2">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="AA79" t="s" s="2">
         <v>20</v>
@@ -11799,10 +11803,10 @@
     </row>
     <row r="80" hidden="true">
       <c r="A80" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B80" t="s" s="2">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="C80" s="2"/>
       <c r="D80" t="s" s="2">
@@ -11919,10 +11923,10 @@
     </row>
     <row r="81" hidden="true">
       <c r="A81" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="B81" t="s" s="2">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="C81" s="2"/>
       <c r="D81" t="s" s="2">

</xml_diff>